<commit_message>
add insights, improvement, and conclusion
</commit_message>
<xml_diff>
--- a/AR-aging-report/Accounts-Receivable.xlsx
+++ b/AR-aging-report/Accounts-Receivable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fanii\Documents\Ajeng\excel-projects\AR-aging-report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{377D3210-D8FE-43A8-AF57-F257BEFCD3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4132F5E1-9CB0-49C0-9390-BDAE9939251D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,9 +28,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1151" r:id="rId6"/>
-    <pivotCache cacheId="1154" r:id="rId7"/>
-    <pivotCache cacheId="1157" r:id="rId8"/>
+    <pivotCache cacheId="1268" r:id="rId6"/>
+    <pivotCache cacheId="1271" r:id="rId7"/>
+    <pivotCache cacheId="1274" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{876F7934-8845-4945-9796-88D515C7AA90}">
@@ -2285,7 +2285,331 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="105">
+  <dxfs count="213">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
     </dxf>
@@ -6280,7 +6604,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000008A-65B2-4358-BC45-4A006D4FBD17}"/>
+              <c16:uniqueId val="{000000A1-65B2-4358-BC45-4A006D4FBD17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6400,7 +6724,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000097-65B2-4358-BC45-4A006D4FBD17}"/>
+              <c16:uniqueId val="{000000A2-65B2-4358-BC45-4A006D4FBD17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6520,7 +6844,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000098-65B2-4358-BC45-4A006D4FBD17}"/>
+              <c16:uniqueId val="{000000A3-65B2-4358-BC45-4A006D4FBD17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6642,7 +6966,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000099-65B2-4358-BC45-4A006D4FBD17}"/>
+              <c16:uniqueId val="{000000A4-65B2-4358-BC45-4A006D4FBD17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6783,7 +7107,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000009A-65B2-4358-BC45-4A006D4FBD17}"/>
+              <c16:uniqueId val="{000000A5-65B2-4358-BC45-4A006D4FBD17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7997,7 +8321,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000030-44F7-418E-A3E9-554CF70DD924}"/>
+              <c16:uniqueId val="{00000047-44F7-418E-A3E9-554CF70DD924}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8074,7 +8398,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000003D-44F7-418E-A3E9-554CF70DD924}"/>
+              <c16:uniqueId val="{00000048-44F7-418E-A3E9-554CF70DD924}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8151,7 +8475,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000003E-44F7-418E-A3E9-554CF70DD924}"/>
+              <c16:uniqueId val="{00000049-44F7-418E-A3E9-554CF70DD924}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8230,7 +8554,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000003F-44F7-418E-A3E9-554CF70DD924}"/>
+              <c16:uniqueId val="{0000004A-44F7-418E-A3E9-554CF70DD924}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8307,7 +8631,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000040-44F7-418E-A3E9-554CF70DD924}"/>
+              <c16:uniqueId val="{0000004B-44F7-418E-A3E9-554CF70DD924}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11271,7 +11595,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000087-EB5C-4EB4-9A62-8C6E2E94A677}"/>
+              <c16:uniqueId val="{0000009E-EB5C-4EB4-9A62-8C6E2E94A677}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11391,7 +11715,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000094-EB5C-4EB4-9A62-8C6E2E94A677}"/>
+              <c16:uniqueId val="{0000009F-EB5C-4EB4-9A62-8C6E2E94A677}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11511,7 +11835,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000095-EB5C-4EB4-9A62-8C6E2E94A677}"/>
+              <c16:uniqueId val="{000000A0-EB5C-4EB4-9A62-8C6E2E94A677}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11633,7 +11957,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000096-EB5C-4EB4-9A62-8C6E2E94A677}"/>
+              <c16:uniqueId val="{000000A1-EB5C-4EB4-9A62-8C6E2E94A677}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11774,7 +12098,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000097-EB5C-4EB4-9A62-8C6E2E94A677}"/>
+              <c16:uniqueId val="{000000A2-EB5C-4EB4-9A62-8C6E2E94A677}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12424,7 +12748,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000030-A1AA-47DE-AC90-ED2ED146E7AC}"/>
+              <c16:uniqueId val="{00000047-A1AA-47DE-AC90-ED2ED146E7AC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12501,7 +12825,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000003D-A1AA-47DE-AC90-ED2ED146E7AC}"/>
+              <c16:uniqueId val="{00000048-A1AA-47DE-AC90-ED2ED146E7AC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12578,7 +12902,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000003E-A1AA-47DE-AC90-ED2ED146E7AC}"/>
+              <c16:uniqueId val="{00000049-A1AA-47DE-AC90-ED2ED146E7AC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12657,7 +12981,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000003F-A1AA-47DE-AC90-ED2ED146E7AC}"/>
+              <c16:uniqueId val="{0000004A-A1AA-47DE-AC90-ED2ED146E7AC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12734,7 +13058,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000040-A1AA-47DE-AC90-ED2ED146E7AC}"/>
+              <c16:uniqueId val="{0000004B-A1AA-47DE-AC90-ED2ED146E7AC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -15126,106 +15450,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1730827</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>146503</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>-1</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>174172</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="monthly!B25">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="Rectangle: Rounded Corners 15">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0B1D957-C03B-0585-A800-406A85C27E49}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2340427" y="1071789"/>
-          <a:ext cx="3842658" cy="1421040"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="accent3">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="accent3"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:endParaRPr lang="en-US" sz="2800" b="1" i="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:fld id="{536249C1-519A-4860-B832-3950B363BD70}" type="TxLink">
-            <a:rPr lang="en-US" sz="2800" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri"/>
-              <a:ea typeface="Calibri"/>
-              <a:cs typeface="Calibri"/>
-            </a:rPr>
-            <a:t>€ 2.385.725,73</a:t>
-          </a:fld>
-          <a:endParaRPr lang="en-GB" sz="2800" b="1">
-            <a:solidFill>
-              <a:schemeClr val="bg1"/>
-            </a:solidFill>
-            <a:effectLst/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>44903</xdr:colOff>
       <xdr:row>13</xdr:row>
@@ -15303,13 +15527,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>371474</xdr:colOff>
+      <xdr:colOff>361950</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>7896</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1790699</xdr:colOff>
+      <xdr:colOff>1781175</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>143422</xdr:rowOff>
     </xdr:to>
@@ -15347,7 +15571,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="371474" y="2696667"/>
+              <a:off x="361950" y="2696667"/>
               <a:ext cx="2028825" cy="1801041"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -15458,16 +15682,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>555171</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>134711</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>25854</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>132897</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>24040</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" Requires="tsle">
@@ -15503,8 +15727,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="7347857" y="1059997"/>
-              <a:ext cx="11952515" cy="1391557"/>
+              <a:off x="361950" y="1136197"/>
+              <a:ext cx="11557907" cy="1391557"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -15535,119 +15759,225 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>108857</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>119743</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>903512</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>168275</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>446314</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>185056</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>10887</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="20" name="Rectangle 19">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="21" name="Group 20">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{072BA57D-A658-DEA2-93DC-EFF9ABA6FC28}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B8A20F59-A944-8AA4-0C52-44B1AAD458A9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2590800" y="1230086"/>
-          <a:ext cx="3429000" cy="402771"/>
+          <a:off x="12587149" y="1093561"/>
+          <a:ext cx="3850278" cy="1421040"/>
+          <a:chOff x="3679369" y="375104"/>
+          <a:chExt cx="3842658" cy="1421040"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-GB" sz="2000" b="0" i="0">
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="monthly!D25">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="16" name="Rectangle: Rounded Corners 15">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0B1D957-C03B-0585-A800-406A85C27E49}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3679369" y="375104"/>
+            <a:ext cx="3842658" cy="1421040"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="accent3">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:endParaRPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:sysClr val="windowText" lastClr="000000"/>
               </a:solidFill>
               <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Outstanding Amount</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-GB" sz="2000">
+              <a:latin typeface="Calibri"/>
+              <a:ea typeface="Calibri"/>
+              <a:cs typeface="Calibri"/>
+            </a:endParaRPr>
+          </a:p>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:fld id="{EA969080-5AD8-408C-ABD1-0B97ECFECF21}" type="TxLink">
+              <a:rPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:pPr algn="ctr"/>
+              <a:t>€ 2.385.725,73</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-GB" sz="3200" b="1">
               <a:solidFill>
                 <a:sysClr val="windowText" lastClr="000000"/>
               </a:solidFill>
               <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-NL" sz="2000">
-            <a:solidFill>
-              <a:sysClr val="windowText" lastClr="000000"/>
-            </a:solidFill>
-            <a:effectLst/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:endParaRPr lang="en-NL" sz="2000">
-            <a:solidFill>
-              <a:sysClr val="windowText" lastClr="000000"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="20" name="Rectangle 19">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{072BA57D-A658-DEA2-93DC-EFF9ABA6FC28}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3864428" y="587829"/>
+            <a:ext cx="3429000" cy="402771"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB" sz="2000" b="0" i="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>Outstanding Amount</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" sz="2000">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t> </a:t>
+            </a:r>
+            <a:endParaRPr lang="en-NL" sz="2000">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:effectLst/>
+            </a:endParaRPr>
+          </a:p>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:endParaRPr lang="en-NL" sz="2000">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -15775,16 +16105,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1226820</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>358140</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:rowOff>129540</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>678180</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>53340</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15811,16 +16141,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>106681</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>175260</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>121921</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>548640</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>38101</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>53341</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -15856,7 +16186,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6957060" y="3764281"/>
+              <a:off x="175260" y="1950721"/>
               <a:ext cx="1828800" cy="1760220"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -15889,16 +16219,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>548640</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>53339</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>236220</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>45719</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -15934,7 +16264,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6957060" y="1988820"/>
+              <a:off x="167640" y="3810000"/>
               <a:ext cx="1828800" cy="1722119"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -15969,7 +16299,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Sabrina Asri" refreshedDate="46064.744681597222" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{EDD2238A-93A9-4D2B-93FE-0C205980EDBA}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Sabrina Asri" refreshedDate="46064.876735763886" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{EDD2238A-93A9-4D2B-93FE-0C205980EDBA}">
   <cacheSource type="external" connectionId="1"/>
   <cacheFields count="4">
     <cacheField name="[Measures].[Sum of outstanding_amount]" caption="Sum of outstanding_amount" numFmtId="0" hierarchy="17" level="32767"/>
@@ -16069,7 +16399,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Sabrina Asri" refreshedDate="46064.744682175929" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{49FC8653-A7A1-4476-8C79-28DE0AEC7A8C}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Sabrina Asri" refreshedDate="46064.876736458333" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{49FC8653-A7A1-4476-8C79-28DE0AEC7A8C}">
   <cacheSource type="external" connectionId="1"/>
   <cacheFields count="3">
     <cacheField name="[AR_table 1].[customer].[customer]" caption="customer" numFmtId="0" hierarchy="1" level="1">
@@ -16151,7 +16481,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Sabrina Asri" refreshedDate="46064.744682986115" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{108F47AE-73C4-42E5-AEFC-C76DF7EEA206}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Sabrina Asri" refreshedDate="46064.876737037041" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{108F47AE-73C4-42E5-AEFC-C76DF7EEA206}">
   <cacheSource type="external" connectionId="1"/>
   <cacheFields count="3">
     <cacheField name="[AR_table 1].[due_date (Month)].[due_date (Month)]" caption="due_date (Month)" numFmtId="0" hierarchy="10" level="1">
@@ -16330,7 +16660,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BE135F79-A040-4F30-BE6D-D2D73E406B17}" name="PivotTable12" cacheId="1151" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BE135F79-A040-4F30-BE6D-D2D73E406B17}" name="PivotTable12" cacheId="1268" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="A3:G26" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -16465,17 +16795,17 @@
     <dataField name="Sum of outstanding_amount" fld="0" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="92">
+    <format dxfId="200">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="93">
+    <format dxfId="201">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="94">
+    <format dxfId="202">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -16646,7 +16976,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3B729F78-C42F-4097-BBC5-D4C810988AD0}" name="PivotTable13" cacheId="1154" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3B729F78-C42F-4097-BBC5-D4C810988AD0}" name="PivotTable13" cacheId="1271" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="A3:G10" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -16719,7 +17049,7 @@
     <dataField name="Sum of outstanding_amount" fld="1" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="95">
+    <format dxfId="203">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -16889,7 +17219,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71179AFE-DAFC-496D-95C8-781976904D54}" name="PivotTable18" cacheId="1157" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71179AFE-DAFC-496D-95C8-781976904D54}" name="PivotTable18" cacheId="1274" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -16995,26 +17325,26 @@
     <dataField name="Sum of outstanding_amount" fld="2" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="8">
-    <format dxfId="91">
+    <format dxfId="199">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="90">
+    <format dxfId="198">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="89">
+    <format dxfId="197">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="88">
+    <format dxfId="196">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="87">
+    <format dxfId="195">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="194">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="0" count="11">
@@ -17036,7 +17366,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="85">
+    <format dxfId="193">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="0" count="8">
@@ -17055,7 +17385,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="192">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -17186,20 +17516,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{427B6372-0638-4E68-BDB0-95989B952CD3}" name="AR_table" displayName="AR_table" ref="A1:G600" totalsRowShown="0" dataDxfId="96" tableBorderDxfId="104">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{427B6372-0638-4E68-BDB0-95989B952CD3}" name="AR_table" displayName="AR_table" ref="A1:G600" totalsRowShown="0" dataDxfId="204" tableBorderDxfId="212">
   <autoFilter ref="A1:G600" xr:uid="{427B6372-0638-4E68-BDB0-95989B952CD3}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{959799F2-B91D-4D60-BE1E-8398A9023901}" name="ar_id" dataDxfId="103"/>
-    <tableColumn id="2" xr3:uid="{04943289-A590-4290-9A75-8E8541C7EC3B}" name="customer" dataDxfId="102"/>
-    <tableColumn id="3" xr3:uid="{4496B90E-A6A6-4848-B8E2-EA4FB5B972EA}" name="invoice_date" dataDxfId="101"/>
-    <tableColumn id="4" xr3:uid="{71EFA1D8-3499-45A7-B6DF-2E87BE1FDD03}" name="due_date" dataDxfId="100">
+    <tableColumn id="1" xr3:uid="{959799F2-B91D-4D60-BE1E-8398A9023901}" name="ar_id" dataDxfId="211"/>
+    <tableColumn id="2" xr3:uid="{04943289-A590-4290-9A75-8E8541C7EC3B}" name="customer" dataDxfId="210"/>
+    <tableColumn id="3" xr3:uid="{4496B90E-A6A6-4848-B8E2-EA4FB5B972EA}" name="invoice_date" dataDxfId="209"/>
+    <tableColumn id="4" xr3:uid="{71EFA1D8-3499-45A7-B6DF-2E87BE1FDD03}" name="due_date" dataDxfId="208">
       <calculatedColumnFormula>WORKDAY(AR_table!$C2,$J$1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{2A9E4D3E-48BF-4103-9329-769E86D1618A}" name="outstanding_amount" dataDxfId="99"/>
-    <tableColumn id="6" xr3:uid="{428956C3-5BCC-40B5-A88C-526B2A897A5B}" name="past_due_days" dataDxfId="98">
+    <tableColumn id="5" xr3:uid="{2A9E4D3E-48BF-4103-9329-769E86D1618A}" name="outstanding_amount" dataDxfId="207"/>
+    <tableColumn id="6" xr3:uid="{428956C3-5BCC-40B5-A88C-526B2A897A5B}" name="past_due_days" dataDxfId="206">
       <calculatedColumnFormula>IF(AR_table!$D2&gt;=TODAY(),0,NETWORKDAYS(AR_table!$D2,TODAY()))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{4C405945-36BE-4C47-869F-DA41572F14F3}" name="aging_category" dataDxfId="97">
+    <tableColumn id="7" xr3:uid="{4C405945-36BE-4C47-869F-DA41572F14F3}" name="aging_category" dataDxfId="205">
       <calculatedColumnFormula>VLOOKUP(AR_table!$F2,aging_bucket[#All],2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -18355,12 +18685,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8140124A-A4C5-45A5-AF39-565715D57464}">
-  <dimension ref="A3:B25"/>
+  <dimension ref="A3:D25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="280" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="280" width="10.77734375" bestFit="1" customWidth="1"/>
     <col min="281" max="281" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -18472,7 +18804,7 @@
       </c>
       <c r="B16" s="2"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="37" t="s">
         <v>616</v>
       </c>
@@ -18480,7 +18812,7 @@
         <v>149106.4</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="37" t="s">
         <v>617</v>
       </c>
@@ -18488,7 +18820,7 @@
         <v>58581.78</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="37" t="s">
         <v>618</v>
       </c>
@@ -18496,7 +18828,7 @@
         <v>72341.59</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="37" t="s">
         <v>619</v>
       </c>
@@ -18504,7 +18836,7 @@
         <v>84319.09</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="37" t="s">
         <v>620</v>
       </c>
@@ -18512,7 +18844,7 @@
         <v>71382.100000000006</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="37" t="s">
         <v>621</v>
       </c>
@@ -18520,7 +18852,7 @@
         <v>101709.6</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="37" t="s">
         <v>622</v>
       </c>
@@ -18528,7 +18860,7 @@
         <v>94829.03</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="37" t="s">
         <v>623</v>
       </c>
@@ -18536,11 +18868,15 @@
         <v>29219.69</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="35" t="s">
         <v>609</v>
       </c>
       <c r="B25" s="2">
+        <v>2385725.73</v>
+      </c>
+      <c r="D25" s="2">
+        <f>GETPIVOTDATA("[Measures].[Sum of outstanding_amount]",$A$3)</f>
         <v>2385725.73</v>
       </c>
     </row>

</xml_diff>